<commit_message>
feat: polish dashboard UI, fix sidebar toggle stacking, add styled auth badges & update README
</commit_message>
<xml_diff>
--- a/backend/income_details.xlsx
+++ b/backend/income_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,35 +415,63 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sdfg</v>
+        <v>h</v>
       </c>
       <c r="B2">
-        <v>54</v>
+        <v>122</v>
       </c>
       <c r="C2" t="str">
         <v>Salary</v>
       </c>
       <c r="D2" t="str">
-        <v>8/5/2026</v>
+        <v>10/4/2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sdfg</v>
+        <v>Sell</v>
       </c>
       <c r="B3">
-        <v>345</v>
+        <v>12</v>
       </c>
       <c r="C3" t="str">
-        <v>Food</v>
+        <v>Salary</v>
       </c>
       <c r="D3" t="str">
-        <v>8/5/2026</v>
+        <v>10/4/2026</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>tjier</v>
+      </c>
+      <c r="B4">
+        <v>12</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="D4" t="str">
+        <v>10/3/2026</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Aalu</v>
+      </c>
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Bonus</v>
+      </c>
+      <c r="D5" t="str">
+        <v>10/3/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>